<commit_message>
docs: renumber tests T01-T19 by priority
</commit_message>
<xml_diff>
--- a/docs/scoring-sheet.xlsx
+++ b/docs/scoring-sheet.xlsx
@@ -550,7 +550,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>填写说明：单项得分只填 100 / 80 / 60 / 0 或 N/A；B 类可填 N/A（自动剔除权重并归一化），A 类（T01–T10）与 C 类（T16–T19）不允许 N/A；权重分布 A 50 / B 20 / C 30；打分依据见 docs/test-procedures.md。</t>
+          <t>编号即优先级（C 类 T01–T04 → B 类 T05–T09 → A 类 T10–T19，权重 C 45 / B 20 / A 35）；单项得分只填 100 / 80 / 60 / 0 或 N/A；B 类（T05–T09）可填 N/A（自动剔除权重并归一化），C 类与 A 类不允许 N/A；打分依据见 docs/test-procedures.md。</t>
         </is>
       </c>
     </row>
@@ -609,16 +609,16 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>单目标定质量</t>
+          <t>排球检测模型精度</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="4">
@@ -643,16 +643,16 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>双目外参标定质量</t>
+          <t>检测推理速度</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="4">
@@ -677,16 +677,16 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>标定重复性</t>
+          <t>动态球测距</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="4">
@@ -711,16 +711,16 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>标定板空间覆盖</t>
+          <t>发球时机与自动击球闭环</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="4">
@@ -745,16 +745,16 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>不同距离深度误差</t>
+          <t>光照鲁棒性</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="4">
@@ -779,12 +779,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>深度精度</t>
+          <t>机械稳定性</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
@@ -813,16 +813,16 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>三轴定位精度</t>
+          <t>温度稳定性</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="4">
@@ -847,16 +847,16 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>极线校正质量</t>
+          <t>时间同步</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="4">
@@ -881,12 +881,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>视差精度</t>
+          <t>动态目标深度精度</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
@@ -915,7 +915,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>目标姿态适应性</t>
+          <t>单目标定质量</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -949,12 +949,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>光照鲁棒性</t>
+          <t>双目外参标定质量</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
@@ -983,16 +983,16 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>机械稳定性</t>
+          <t>标定重复性</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="4">
@@ -1017,12 +1017,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>温度稳定性</t>
+          <t>标定板空间覆盖</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
@@ -1051,16 +1051,16 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>时间同步</t>
+          <t>不同距离深度误差</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="4">
@@ -1085,16 +1085,16 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>动态目标深度精度</t>
+          <t>深度精度</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="4">
@@ -1119,16 +1119,16 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>排球检测模型精度</t>
+          <t>三轴定位精度</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="4">
@@ -1153,16 +1153,16 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>检测推理速度</t>
+          <t>极线校正质量</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="4">
@@ -1187,16 +1187,16 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>动态球测距</t>
+          <t>视差精度</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="4">
@@ -1221,16 +1221,16 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>发球时机与自动击球闭环</t>
+          <t>目标姿态适应性</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="4">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>合计（A 50 / B 20 / C 30）</t>
+          <t>合计（C 45 / B 20 / A 35）</t>
         </is>
       </c>
       <c r="C23" s="9" t="n"/>
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>IF(B26="是","F",IF(NOT(ISNUMBER(B25)),"",IF(AND(B25&gt;=90,COUNT(E4:E13)=10),"A",IF(B25&gt;=80,"B",IF(AND(B25&gt;=70,COUNTIF(E4:E13,0)=0),"C","F")))))</f>
+        <f>IF(B26="是","F",IF(NOT(ISNUMBER(B25)),"",IF(AND(B25&gt;=90,COUNT(E13:E22)=10,COUNT(E4:E7)=4),"A",IF(B25&gt;=80,"B",IF(AND(B25&gt;=70,COUNTIF(E13:E22,0)=0,COUNTIF(E4:E7,0)=0),"C","F")))))</f>
         <v/>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>T01 单目重投影 RMS 或 T02 双目重投影 RMS 落在"不合格"档</t>
+          <t>T10 单目重投影 RMS 或 T11 双目重投影 RMS 落在"不合格"档</t>
         </is>
       </c>
       <c r="C3" s="4" t="n"/>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>T08 极线误差 RMS 超过合格档（&gt; 0.50 px）</t>
+          <t>T17 极线误差 RMS 超过合格档（&gt; 0.50 px）</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>T12 触发"标定失效"判据（ΔB/B 或 ΔR 任一超合格档）</t>
+          <t>T06 机械稳定性触发"标定失效"判据（ΔB/B 或 ΔR 任一超合格档）</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>

</xml_diff>